<commit_message>
Refactor: rename Scenario to ImplOption (实现选项) globally
</commit_message>
<xml_diff>
--- a/templates/soc_import_template.xlsx
+++ b/templates/soc_import_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="module_definitions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="projects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="scenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="implOptions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="tiers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="logical_components" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="physical_partitions" sheetId="7" state="visible" r:id="rId7"/>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'instructions'!$A$1:$B$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'module_definitions'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'projects'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'scenarios'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'implOptions'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'tiers'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'logical_components'!$A$1:$K$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'physical_partitions'!$A$1:$J$9</definedName>
@@ -180,7 +180,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="coverage_checks_table" displayName="coverage_checks_table" ref="A1:H6" headerRowCount="1">
   <autoFilter ref="A1:H6"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="scenario_id"/>
+    <tableColumn id="1" name="impl_option_id"/>
     <tableColumn id="2" name="logical_component_id"/>
     <tableColumn id="3" name="resource_category"/>
     <tableColumn id="4" name="logical_name"/>
@@ -209,13 +209,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="scenarios_table" displayName="scenarios_table" ref="A1:F2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="implOptions_table" displayName="implOptions_table" ref="A1:F2" headerRowCount="1">
   <autoFilter ref="A1:F2"/>
   <tableColumns count="6">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="project_id"/>
     <tableColumn id="3" name="name"/>
-    <tableColumn id="4" name="scenario_type"/>
+    <tableColumn id="4" name="impl_type"/>
     <tableColumn id="5" name="process_combo"/>
     <tableColumn id="6" name="status"/>
   </tableColumns>
@@ -228,7 +228,7 @@
   <autoFilter ref="A1:H4"/>
   <tableColumns count="8">
     <tableColumn id="1" name="id"/>
-    <tableColumn id="2" name="scenario_id"/>
+    <tableColumn id="2" name="impl_option_id"/>
     <tableColumn id="3" name="tier_index"/>
     <tableColumn id="4" name="name"/>
     <tableColumn id="5" name="process_id"/>
@@ -265,7 +265,7 @@
   <autoFilter ref="A1:J9"/>
   <tableColumns count="10">
     <tableColumn id="1" name="id"/>
-    <tableColumn id="2" name="scenario_id"/>
+    <tableColumn id="2" name="impl_option_id"/>
     <tableColumn id="3" name="logical_component_id"/>
     <tableColumn id="4" name="tier_id"/>
     <tableColumn id="5" name="partition_name"/>
@@ -284,7 +284,7 @@
   <autoFilter ref="A1:N18"/>
   <tableColumns count="14">
     <tableColumn id="1" name="id"/>
-    <tableColumn id="2" name="scenario_id"/>
+    <tableColumn id="2" name="impl_option_id"/>
     <tableColumn id="3" name="subject_type"/>
     <tableColumn id="4" name="subject_id"/>
     <tableColumn id="5" name="metric_name"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Minimal physical partition table from logical components to scenario/tier placement. resource_category splits logic, SRAM, and block/hard-macro content. Details live in metrics.</t>
+          <t>Minimal physical partition table from logical components to impl_option/tier placement. resource_category splits logic, SRAM, and block/hard-macro content. Details live in metrics.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Unified metric table. Metrics can attach to logical_component, physical_partition, tier, or scenario.</t>
+          <t>Unified metric table. Metrics can attach to logical_component, physical_partition, tier, or impl_option.</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The same metric_name can appear at logical_component, physical_partition, tier, or scenario level; subject_type defines meaning.</t>
+          <t>The same metric_name can appear at logical_component, physical_partition, tier, or impl_option level; subject_type defines meaning.</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -998,7 +998,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>scenario_id</t>
+          <t>impl_option_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>scenario_type</t>
+          <t>impl_type</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1612,7 +1612,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>scenario_id</t>
+          <t>impl_option_id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2202,7 +2202,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>scenario_id</t>
+          <t>impl_option_id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2676,7 +2676,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>scenario_id</t>
+          <t>impl_option_id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3884,7 +3884,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>M_SCENARIO_AREA</t>
+          <t>M_IMPL_OPTION_AREA</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>scenario</t>
+          <t>impl_option</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Scenario-level summary estimate.</t>
+          <t>ImplOption-level summary estimate.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -3955,7 +3955,7 @@
   <autoFilter ref="A1:N18"/>
   <dataValidations count="3">
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"logical_component,physical_partition,tier,scenario"</formula1>
+      <formula1>"logical_component,physical_partition,tier,impl_option"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"number,text,boolean"</formula1>
@@ -4171,12 +4171,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>tier,scenario</t>
+          <t>tier,impl_option</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Tier or scenario area estimate. Logical modules and physical partitions use logic_area/sram_area/block_area.</t>
+          <t>Tier or impl_option area estimate. Logical modules and physical partitions use logic_area/sram_area/block_area.</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>logical_component,physical_partition,tier,scenario</t>
+          <t>logical_component,physical_partition,tier,impl_option</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fix duplicate hierarchy path cleanup
</commit_message>
<xml_diff>
--- a/templates/soc_import_template.xlsx
+++ b/templates/soc_import_template.xlsx
@@ -1792,7 +1792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1915,7 +1915,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B30</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1925,48 +1925,52 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>B0</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
+          <t>B_NPU</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>MD_NPU_MAC</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NPU_TOP</t>
+          <t>NPU_MAC_ARRAY</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>subsystem</t>
+          <t>block</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>logic+memory</t>
+          <t>logic</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>AI Compute</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>SOC_TOP/NPU_TOP</t>
+          <t>SOC_TOP/NPU_TOP/NPU_MAC_ARRAY</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>NPU subsystem containing repeated MAC and SRAM modules.</t>
+          <t>Logical MAC array module. Repetition is captured by logical_instance_count.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1976,52 +1980,52 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B_NPU</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>MD_NPU_MAC</t>
+          <t>MD_NPU_SRAM</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NPU_MAC_ARRAY</t>
+          <t>NPU_SRAM_BANK</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>block</t>
+          <t>macro_group</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>logic</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>AI Compute</t>
+          <t>AI Memory</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>SOC_TOP/NPU_TOP/NPU_MAC_ARRAY</t>
+          <t>SOC_TOP/NPU_TOP/NPU_SRAM_BANK</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Logical MAC array module. Repetition is captured by logical_instance_count.</t>
+          <t>Logical SRAM bank module.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2031,153 +2035,43 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B0</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>MD_NPU_SRAM</t>
+          <t>MD_DDR_PHY</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>NPU_SRAM_BANK</t>
+          <t>DDR_PHY</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>macro_group</t>
+          <t>phy</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>phy_analog</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>AI Memory</t>
+          <t>Memory IO</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>SOC_TOP/NPU_TOP/NPU_SRAM_BANK</t>
+          <t>SOC_TOP/DDR_PHY</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Logical SRAM bank module.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>B0</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>MD_GPU_TOP</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>GPU_TOP</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>subsystem</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>logic+memory</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Graphics</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>SOC_TOP/GPU_TOP</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>GPU logical module may be partially partitioned across tiers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>B5</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>B0</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>MD_DDR_PHY</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>DDR_PHY</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>phy</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>phy_analog</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Memory IO</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>SOC_TOP/DDR_PHY</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Fixed bottom-tier PHY.</t>
         </is>
@@ -2518,7 +2412,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B_GPU</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2566,7 +2460,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B_GPU</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove legacy redundant NPU children
</commit_message>
<xml_diff>
--- a/templates/soc_import_template.xlsx
+++ b/templates/soc_import_template.xlsx
@@ -1792,7 +1792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1915,7 +1915,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1925,153 +1925,43 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>B_NPU</t>
+          <t>B0</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>MD_NPU_MAC</t>
+          <t>MD_DDR_PHY</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NPU_MAC_ARRAY</t>
+          <t>DDR_PHY</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>block</t>
+          <t>phy</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>logic</t>
+          <t>phy_analog</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>AI Compute</t>
+          <t>Memory IO</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>SOC_TOP/NPU_TOP/NPU_MAC_ARRAY</t>
+          <t>SOC_TOP/DDR_PHY</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Logical MAC array module. Repetition is captured by logical_instance_count.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>B_NPU</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>MD_NPU_SRAM</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>NPU_SRAM_BANK</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>macro_group</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>AI Memory</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>SOC_TOP/NPU_TOP/NPU_SRAM_BANK</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Logical SRAM bank module.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>B5</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>B0</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>MD_DDR_PHY</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>DDR_PHY</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>phy</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>phy_analog</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Memory IO</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>SOC_TOP/DDR_PHY</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Fixed bottom-tier PHY.</t>
         </is>
@@ -2092,7 +1982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2162,7 +2052,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PP_NPU_MAC_ARRAY_logic_T0</t>
+          <t>PP_GPU_TOP_logic_T0_P1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2172,7 +2062,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>B_GPU</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2182,7 +2072,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>NPU_MAC_ARRAY_logic_T0</t>
+          <t>GPU_TOP_logic_T0_P1</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -2192,25 +2082,25 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>All four MAC logic copies are implemented on the top tier.</t>
+          <t>GPU residual/self logic-side partition on top tier.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PP_NPU_MAC_ARRAY_block_T0</t>
+          <t>PP_GPU_TOP_logic_T1_P2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2220,45 +2110,45 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>B_GPU</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>T0</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NPU_MAC_ARRAY_block_T0</t>
+          <t>GPU_TOP_logic_T1_P2</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>block</t>
+          <t>logic</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>All four MAC block-area copies are implemented on the top tier.</t>
+          <t>GPU residual/self logic-side partition on memory tier.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PP_NPU_SRAM_BANK_logic_T1</t>
+          <t>PP_DDR_PHY_block_T2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2268,22 +2158,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NPU_SRAM_BANK_logic_T1</t>
+          <t>DDR_PHY_block_T2</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>logic</t>
+          <t>block</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2292,252 +2182,12 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>SRAM peripheral/control logic on the memory tier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_SRAM_BANK_sram_T1</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>NPU_SRAM_BANK_sram_T1</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>sram</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>full</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Both logical SRAM bank copies are carried by this middle-tier partition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_SRAM_BANK_block_T1</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>NPU_SRAM_BANK_block_T1</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>block</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>full</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Block-level SRAM-bank implementation area on the memory tier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>PP_GPU_TOP_logic_T0_P1</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>B_GPU</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>T0</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>GPU_TOP_logic_T0_P1</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>logic</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>GPU residual/self logic-side partition on top tier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>PP_GPU_TOP_logic_T1_P2</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>B_GPU</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>GPU_TOP_logic_T1_P2</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>logic</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>GPU residual/self logic-side partition on memory tier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>PP_DDR_PHY_block_T2</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>B5</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>DDR_PHY_block_T2</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>block</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>full</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Fixed PHY hard/block content on bottom tier.</t>
         </is>
@@ -2566,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2660,7 +2310,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>M_LOG_B30_SIGNALS</t>
+          <t>M_PART_GPU_LOGIC_AREA_TOP</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2670,30 +2320,30 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>logical_component</t>
+          <t>physical_partition</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>PP_GPU_TOP_logic_T0_P1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>signal_count_total</t>
+          <t>logic_area</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mm2</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>logical</t>
+          <t>implementation_area</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2718,7 +2368,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Total logical signal count. Input/output/inout are intentionally not split in phase 1.</t>
+          <t>Logic-side area for GPU top-tier partition.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -2730,7 +2380,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M_LOG_B30_LOGIC_AREA</t>
+          <t>M_PART_GPU_LOGIC_AREA_MID</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2740,12 +2390,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>logical_component</t>
+          <t>physical_partition</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>PP_GPU_TOP_logic_T1_P2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2754,7 +2404,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10.6</v>
+        <v>6.7</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -2763,7 +2413,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>logical_area</t>
+          <t>implementation_area</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2788,7 +2438,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Logic area estimate for all four MAC instances.</t>
+          <t>Logic-side area for GPU middle-tier partition.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -2800,7 +2450,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M_LOG_B30_SRAM_AREA</t>
+          <t>M_PART_GPU_LOGIC_POWER</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2810,30 +2460,30 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>logical_component</t>
+          <t>physical_partition</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>PP_GPU_TOP_logic_T0_P1</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sram_area</t>
+          <t>power</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>mm2</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>logical_area</t>
+          <t>power</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2848,7 +2498,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>nominal</t>
+          <t>peak</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -2858,7 +2508,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>SRAM area estimate for all four MAC instances.</t>
+          <t>Power estimate for GPU logic partition.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2870,7 +2520,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>M_LOG_B30_BLOCK_AREA</t>
+          <t>M_TIER_T0_POWER</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2880,30 +2530,30 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>logical_component</t>
+          <t>tier</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>block_area</t>
+          <t>power</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.8</v>
+        <v>7.6</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>mm2</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>logical_area</t>
+          <t>power</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -2918,7 +2568,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>nominal</t>
+          <t>peak</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -2928,7 +2578,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Block area estimate including logic, SRAM, and early overhead.</t>
+          <t>Tier-level rollup or target.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2940,7 +2590,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>M_LOG_B8_SIGNALS</t>
+          <t>M_IMPL_OPTION_AREA</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -2950,30 +2600,30 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>logical_component</t>
+          <t>impl_option</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>signal_count_total</t>
+          <t>area</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>24</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mm2</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>logical</t>
+          <t>physical</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2998,848 +2648,10 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Total logical signal count for SRAM bank module.</t>
+          <t>ImplOption-level summary estimate.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>M_LOG_B8_LOGIC_AREA</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>logical_component</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>logic_area</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>logical_area</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Peripheral/control logic area.</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>M_LOG_B8_SRAM_AREA</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>logical_component</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>sram_area</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>logical_area</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>SRAM macro area estimate.</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>M_LOG_B8_BLOCK_AREA</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>logical_component</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>block_area</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>logical_area</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Block area estimate including early overhead.</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_MAC_LOGIC_AREA</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_MAC_ARRAY_logic_T0</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>logic_area</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>implementation_area</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Implementation-level logic area for MAC logic partition.</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_MAC_LOGIC_SHAPE</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_MAC_ARRAY_logic_T0</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>shape_type</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>logic_array</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>physical_shape</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>Optional shape descriptor, kept out of physical_partitions.</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_MAC_BLOCK_AREA</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_MAC_ARRAY_block_T0</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>block_area</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>implementation_area</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Implementation block area for MAC array.</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_SRAM_SRAM_AREA</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>PP_NPU_SRAM_BANK_sram_T1</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>sram_area</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>implementation_area</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>SRAM area for NPU SRAM bank partition.</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_GPU_LOGIC_AREA_TOP</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>PP_GPU_TOP_logic_T0_P1</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>logic_area</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>implementation_area</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>Logic-side area for GPU top-tier partition.</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_GPU_LOGIC_AREA_MID</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>PP_GPU_TOP_logic_T1_P2</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>logic_area</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>implementation_area</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Logic-side area for GPU middle-tier partition.</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>M_PART_GPU_LOGIC_POWER</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>physical_partition</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>PP_GPU_TOP_logic_T0_P1</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>power</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>power</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Power estimate for GPU logic partition.</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>M_TIER_T0_POWER</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>tier</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>T0</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>power</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>power</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Tier-level rollup or target.</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>M_IMPL_OPTION_AREA</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>impl_option</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>area</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>physical</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>typical</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>nominal</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>ImplOption-level summary estimate.</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>2026-05-27</t>
         </is>

</xml_diff>